<commit_message>
filter, report DevicesErrors, refactor, tuning
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_device/en.xlsx
+++ b/api/templates/critical_errors_by_device/en.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="71">
   <si>
     <t>Other Error</t>
   </si>
@@ -182,30 +182,9 @@
     <t>&lt;Table&gt;</t>
   </si>
   <si>
-    <t>&lt;#&gt;</t>
-  </si>
-  <si>
-    <t>&lt;deviceName&gt;</t>
-  </si>
-  <si>
     <t>&lt;serial&gt;</t>
   </si>
   <si>
-    <t>&lt;lastUpload&gt;</t>
-  </si>
-  <si>
-    <t>&lt;totalTests&gt;</t>
-  </si>
-  <si>
-    <t>&lt;invalid&gt;</t>
-  </si>
-  <si>
-    <t>&lt;errors&gt;</t>
-  </si>
-  <si>
-    <t>&lt;errorPercentage&gt;</t>
-  </si>
-  <si>
     <t>Errors by Device</t>
   </si>
   <si>
@@ -215,9 +194,6 @@
     <t>States: &lt;States&gt;</t>
   </si>
   <si>
-    <t>County: &lt;County&gt;</t>
-  </si>
-  <si>
     <t>Device</t>
   </si>
   <si>
@@ -227,25 +203,37 @@
     <t>Last Upload</t>
   </si>
   <si>
-    <t>Invalid</t>
-  </si>
-  <si>
-    <t>Errors</t>
-  </si>
-  <si>
     <t>Error Percentage</t>
   </si>
   <si>
     <t>Total Tests Run During Period</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Subtotal for devices not assigned to a state</t>
-  </si>
-  <si>
-    <t>Subtotal for &lt;GeographyName&gt;</t>
+    <t>LGA: &lt;Lgas&gt;</t>
+  </si>
+  <si>
+    <t>&lt;name&gt;</t>
+  </si>
+  <si>
+    <t>&lt;lastUploadOn&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalErrors&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalInvalid&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalResults&gt;</t>
+  </si>
+  <si>
+    <t>&lt;errorRate&gt;</t>
+  </si>
+  <si>
+    <t># Invalid</t>
+  </si>
+  <si>
+    <t># Errors</t>
   </si>
 </sst>
 </file>
@@ -315,7 +303,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -354,10 +342,40 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color auto="1"/>
       </left>
       <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
         <color auto="1"/>
       </right>
       <top style="thin">
@@ -372,10 +390,10 @@
       <left style="medium">
         <color auto="1"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color auto="1"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color auto="1"/>
       </top>
       <bottom style="medium">
@@ -390,68 +408,10 @@
       <right style="medium">
         <color auto="1"/>
       </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
       <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
         <color auto="1"/>
       </top>
       <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -502,7 +462,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="226">
+  <cellXfs count="227">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -512,654 +472,659 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1542,42 +1507,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.125" customWidth="1"/>
-    <col min="2" max="2" width="15.25" customWidth="1"/>
+    <col min="1" max="1" width="31.875" customWidth="1"/>
+    <col min="2" max="2" width="26.375" customWidth="1"/>
     <col min="3" max="3" width="18.125" customWidth="1"/>
-    <col min="4" max="4" width="15" style="204" customWidth="1"/>
+    <col min="4" max="4" width="16.5" style="204" customWidth="1"/>
     <col min="5" max="5" width="11" style="204" customWidth="1"/>
     <col min="6" max="6" width="11" style="204"/>
-    <col min="7" max="7" width="17" style="204" customWidth="1"/>
+    <col min="7" max="7" width="15" style="225" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="217" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B1" s="217"/>
       <c r="C1" s="216"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="216" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B2" s="216"/>
       <c r="C2" s="216"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="216" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B3" s="216"/>
       <c r="C3" s="216"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="216" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B4" s="216"/>
       <c r="C4" s="216"/>
@@ -1594,137 +1559,50 @@
       <c r="B6" s="216"/>
       <c r="C6" s="216"/>
     </row>
-    <row r="7" spans="1:7" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="221" t="s">
+    <row r="7" spans="1:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="218" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="218" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="218" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="219" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="220" t="s">
+        <v>69</v>
+      </c>
+      <c r="F7" s="220" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="226" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="221" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="221" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="222" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="223" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="223" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="223" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="221" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="221" t="s">
-        <v>67</v>
-      </c>
-      <c r="D7" s="222" t="s">
-        <v>71</v>
-      </c>
-      <c r="E7" s="223" t="s">
+      <c r="G8" s="224" t="s">
         <v>68</v>
-      </c>
-      <c r="F7" s="223" t="s">
-        <v>69</v>
-      </c>
-      <c r="G7" s="223" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="218" t="s">
-        <v>54</v>
-      </c>
-      <c r="B8" s="219" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="220" t="s">
-        <v>56</v>
-      </c>
-      <c r="D8" s="224" t="s">
-        <v>57</v>
-      </c>
-      <c r="E8" s="224" t="s">
-        <v>58</v>
-      </c>
-      <c r="F8" s="224" t="s">
-        <v>59</v>
-      </c>
-      <c r="G8" s="225" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="218"/>
-      <c r="B9" s="219"/>
-      <c r="C9" s="220"/>
-      <c r="D9" s="224"/>
-      <c r="E9" s="224"/>
-      <c r="F9" s="224"/>
-      <c r="G9" s="225"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="218"/>
-      <c r="B10" s="219"/>
-      <c r="C10" s="220"/>
-      <c r="D10" s="224"/>
-      <c r="E10" s="224"/>
-      <c r="F10" s="224"/>
-      <c r="G10" s="225"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="218" t="s">
-        <v>73</v>
-      </c>
-      <c r="B11" s="219"/>
-      <c r="C11" s="220"/>
-      <c r="D11" s="224" t="s">
-        <v>53</v>
-      </c>
-      <c r="E11" s="224" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" s="224" t="s">
-        <v>53</v>
-      </c>
-      <c r="G11" s="225" t="e">
-        <f>IF(D11=0,0,(F11)/D11)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="218" t="s">
-        <v>74</v>
-      </c>
-      <c r="B12" s="219"/>
-      <c r="C12" s="220"/>
-      <c r="D12" s="224" t="s">
-        <v>53</v>
-      </c>
-      <c r="E12" s="224" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="224" t="s">
-        <v>53</v>
-      </c>
-      <c r="G12" s="225" t="e">
-        <f>IF(D12=0,0,(F12)/D12)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="218"/>
-      <c r="B13" s="219"/>
-      <c r="C13" s="220"/>
-      <c r="D13" s="224"/>
-      <c r="E13" s="224"/>
-      <c r="F13" s="224"/>
-      <c r="G13" s="225"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="218" t="s">
-        <v>72</v>
-      </c>
-      <c r="B14" s="219"/>
-      <c r="C14" s="220"/>
-      <c r="D14" s="224" t="s">
-        <v>53</v>
-      </c>
-      <c r="E14" s="224" t="s">
-        <v>53</v>
-      </c>
-      <c r="F14" s="224" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" s="225" t="e">
-        <f>IF(D14=0,0,(F14)/D14)</f>
-        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
All reports show state and lga country labels
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_device/en.xlsx
+++ b/api/templates/critical_errors_by_device/en.xlsx
@@ -1,22 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="22730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\critical_errors_by_device\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nicolas\Trabajo\SystemOne\Repositorios\Aspect2\aspect\api\templates\critical_errors_by_device\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9411D1FA-92B5-4BDE-BE3E-7D52BE0BEA4A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6465" tabRatio="815"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Errors by Device" sheetId="1" r:id="rId1"/>
     <sheet name="Error Codes by Device" sheetId="2" r:id="rId2"/>
     <sheet name="Error Codes" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913" fullPrecision="0"/>
+  <calcPr calcId="191029" fullPrecision="0"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -191,9 +202,6 @@
     <t>Dates: &lt;Dates&gt;</t>
   </si>
   <si>
-    <t>States: &lt;States&gt;</t>
-  </si>
-  <si>
     <t>Device</t>
   </si>
   <si>
@@ -209,9 +217,6 @@
     <t>Total Tests Run During Period</t>
   </si>
   <si>
-    <t>LGA: &lt;Lgas&gt;</t>
-  </si>
-  <si>
     <t>&lt;name&gt;</t>
   </si>
   <si>
@@ -234,12 +239,18 @@
   </si>
   <si>
     <t># Errors</t>
+  </si>
+  <si>
+    <t>&lt;State_Label&gt;: &lt;States&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Lga_Label&gt;: &lt;Lgas&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
@@ -1506,7 +1517,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1535,14 +1546,14 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="216" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="B3" s="216"/>
       <c r="C3" s="216"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="216" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B4" s="216"/>
       <c r="C4" s="216"/>
@@ -1561,48 +1572,48 @@
     </row>
     <row r="7" spans="1:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="218" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="218" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="218" t="s">
+      <c r="C7" s="218" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="218" t="s">
+      <c r="D7" s="219" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" s="220" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="220" t="s">
+        <v>68</v>
+      </c>
+      <c r="G7" s="226" t="s">
         <v>59</v>
-      </c>
-      <c r="D7" s="219" t="s">
-        <v>61</v>
-      </c>
-      <c r="E7" s="220" t="s">
-        <v>69</v>
-      </c>
-      <c r="F7" s="220" t="s">
-        <v>70</v>
-      </c>
-      <c r="G7" s="226" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="221" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B8" s="221" t="s">
         <v>53</v>
       </c>
       <c r="C8" s="222" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="223" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" s="223" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="223" t="s">
-        <v>67</v>
-      </c>
-      <c r="E8" s="223" t="s">
+      <c r="F8" s="223" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" s="224" t="s">
         <v>66</v>
-      </c>
-      <c r="F8" s="223" t="s">
-        <v>65</v>
-      </c>
-      <c r="G8" s="224" t="s">
-        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1612,7 +1623,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N18"/>
   <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2250,7 +2261,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
Add error codes sheets in Critical Errors By Device Report
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_device/en.xlsx
+++ b/api/templates/critical_errors_by_device/en.xlsx
@@ -5,10 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Errors by Device" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Error Codes by Device" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Error Codes" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="70">
   <si>
     <t xml:space="preserve">Errors by Device</t>
   </si>
@@ -80,18 +82,169 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;errorRate&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error Codes by Device</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type of error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid Results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total errors, invalid results, no results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;error_5011&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;error_5007&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;error_5006&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;error_2008&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;error_2005&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;error_2037&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;error_2025&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;error_2022&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;mtbNoResult&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;mtbInvalid&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;total&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run-time error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The actual temperature has drifted too far away from the setpoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The temperature difference exceeds the limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The internal instrument temperature was out of range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optic signal of from detector exceeded the limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detector dark signal exceeded the limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The power supply was detected to be out of range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The measured temperature of the optical system was not within the acceptable range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A valve positioning error was detected at the end of the run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operation terminated error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Module is already running a test while performing command</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motion of the syringe drive was not detected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Syringe pressure reading exceeds the protocol limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Syringe pressure reading is below the protocol limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartridge loading error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unable to initialize pressure sensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The digital temperature reading for Thermistor A/Thermistor B/Ambient Thermistor/Optic Thermistor was not within the acceptable range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The system was unable to find the valve home position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt to load a cartridge while the door is still closed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failed to get to desired temperature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The system failed to find the plunger home position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The ultrasonic horn could not be tuned properly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The optical signal from Detector did not reach the expected value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The cartridge integrity test failed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-test error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cooling fan operation was not verified. Measured temperature exceeded the limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post-run analysis error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe check failed. Probe check value was above the maximum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probe check failed. Probe check value was below the minimum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signal loss detected in the amplification curve</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
     <numFmt numFmtId="166" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy;@"/>
+    <numFmt numFmtId="167" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -123,8 +276,22 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -144,7 +311,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -156,6 +323,34 @@
       <left style="medium"/>
       <right style="medium"/>
       <top style="medium"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="medium"/>
+      <top style="thin"/>
       <bottom style="medium"/>
       <diagonal/>
     </border>
@@ -185,7 +380,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -206,23 +401,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -240,6 +435,38 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -320,10 +547,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultColWidth="11.015625" defaultRowHeight="15.6" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15.6" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.4"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="11"/>
@@ -358,7 +585,7 @@
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
     </row>
-    <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
@@ -432,4 +659,515 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr defaultColWidth="9.38671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="33.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="33.12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>5011</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>5007</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>5006</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>2008</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>2005</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>2037</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I9" s="15" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="J10" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="K10" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="L10" s="19" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr defaultColWidth="9.38671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="120.07"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="21" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="21" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="21" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="n">
+        <v>1017</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="n">
+        <v>1018</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="n">
+        <v>2037</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="21" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="n">
+        <v>4010</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21" t="n">
+        <v>4017</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21" t="n">
+        <v>5006</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="n">
+        <v>5007</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21" t="n">
+        <v>5011</v>
+      </c>
+      <c r="B27" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add other error column in Critical Errors by Device report
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_device/en.xlsx
+++ b/api/templates/critical_errors_by_device/en.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="72">
   <si>
     <t xml:space="preserve">Errors by Device</t>
   </si>
@@ -93,6 +93,9 @@
     <t xml:space="preserve">Type of error</t>
   </si>
   <si>
+    <t xml:space="preserve">Other Error</t>
+  </si>
+  <si>
     <t xml:space="preserve">No Results</t>
   </si>
   <si>
@@ -124,6 +127,9 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;error_2022&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;error_other&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;mtbNoResult&gt;</t>
@@ -244,7 +250,7 @@
     <numFmt numFmtId="166" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy;@"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -274,12 +280,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -401,23 +401,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -437,7 +437,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -461,7 +461,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -547,13 +547,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15.6" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.08984375" defaultRowHeight="15.6" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.4"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="15"/>
   </cols>
   <sheetData>
@@ -666,13 +666,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultColWidth="9.38671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultColWidth="9.40234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="33.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="33.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="11.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="33.12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -690,6 +690,7 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
@@ -706,6 +707,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
@@ -722,6 +724,7 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
@@ -740,6 +743,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -758,6 +762,7 @@
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
@@ -798,8 +803,11 @@
       <c r="K9" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="L9" s="16" t="s">
+      <c r="L9" s="15" t="s">
         <v>25</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -807,37 +815,40 @@
         <v>13</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I10" s="17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J10" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="K10" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="L10" s="19" t="s">
+      <c r="K10" s="17" t="s">
         <v>36</v>
+      </c>
+      <c r="L10" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="M10" s="19" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -857,7 +868,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="9.38671875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.40234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.79"/>
@@ -866,13 +877,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -880,10 +891,10 @@
         <v>1001</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -891,10 +902,10 @@
         <v>1002</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -902,10 +913,10 @@
         <v>1004</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -913,10 +924,10 @@
         <v>1005</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -924,10 +935,10 @@
         <v>1006</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -935,10 +946,10 @@
         <v>1007</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -946,10 +957,10 @@
         <v>1017</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -957,10 +968,10 @@
         <v>1018</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -968,10 +979,10 @@
         <v>2003</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -979,10 +990,10 @@
         <v>2005</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -990,10 +1001,10 @@
         <v>2008</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1001,10 +1012,10 @@
         <v>2009</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1012,10 +1023,10 @@
         <v>2011</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1023,10 +1034,10 @@
         <v>2014</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1034,10 +1045,10 @@
         <v>2016</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1045,10 +1056,10 @@
         <v>2018</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1056,10 +1067,10 @@
         <v>2022</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1067,10 +1078,10 @@
         <v>2025</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1078,10 +1089,10 @@
         <v>2032</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1089,10 +1100,10 @@
         <v>2034</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1100,10 +1111,10 @@
         <v>2037</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1111,10 +1122,10 @@
         <v>4010</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1122,10 +1133,10 @@
         <v>4017</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1133,10 +1144,10 @@
         <v>5006</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1144,10 +1155,10 @@
         <v>5007</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1155,10 +1166,10 @@
         <v>5011</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[feat/ASP-7977-Device-Name-Redesign] Reviewed all the modified reports
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_device/en.xlsx
+++ b/api/templates/critical_errors_by_device/en.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2DB8257-9F3B-8E4B-952F-20D6243CEF8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FB26F9E-D018-FF4A-8D67-1516CAA4D466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="80">
   <si>
     <t>Errors by Device</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>Type of error</t>
   </si>
   <si>
     <t>Other Error</t>
@@ -411,7 +408,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1" shrinkToFit="1"/>
@@ -483,6 +480,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,7 +709,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.33203125" customWidth="1"/>
     <col min="4" max="4" width="18.1640625" customWidth="1"/>
     <col min="5" max="5" width="16.5" customWidth="1"/>
@@ -805,10 +812,10 @@
     </row>
     <row r="8" spans="1:14" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>7</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>8</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>9</v>
@@ -849,10 +856,10 @@
     </row>
     <row r="9" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>18</v>
@@ -3172,10 +3179,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="3"/>
+      <c r="B1" s="26"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
@@ -3189,10 +3196,10 @@
       <c r="M1" s="3"/>
     </row>
     <row r="2" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="26"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
@@ -3206,10 +3213,10 @@
       <c r="M2" s="3"/>
     </row>
     <row r="3" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
+      <c r="B3" s="26"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -3223,10 +3230,10 @@
       <c r="M3" s="3"/>
     </row>
     <row r="4" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="26" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="3"/>
@@ -3242,12 +3249,14 @@
       <c r="M4" s="3"/>
     </row>
     <row r="5" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B5" s="28"/>
     </row>
     <row r="6" spans="1:14" ht="16" x14ac:dyDescent="0.2">
-      <c r="B6" s="3"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="26"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -3260,17 +3269,18 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row r="8" spans="1:14" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:14" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="21" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="22"/>
+    </row>
+    <row r="9" spans="1:14" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" s="17">
         <v>5011</v>
@@ -3297,54 +3307,54 @@
         <v>2022</v>
       </c>
       <c r="K9" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="L9" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="L9" s="17" t="s">
+      <c r="M9" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="M9" s="17" t="s">
+      <c r="N9" s="17" t="s">
         <v>35</v>
-      </c>
-      <c r="N9" s="17" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="13" t="s">
+      <c r="D10" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="E10" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="F10" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="G10" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="H10" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="I10" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="J10" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="13" t="s">
+      <c r="K10" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="K10" s="13" t="s">
+      <c r="L10" s="13" t="s">
         <v>46</v>
-      </c>
-      <c r="L10" s="13" t="s">
-        <v>47</v>
       </c>
       <c r="M10" s="13" t="s">
         <v>23</v>
@@ -3354,986 +3364,986 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="116" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="117" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="118" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="119" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="120" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="121" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="122" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="123" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="124" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="125" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="126" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="127" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="128" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="129" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="130" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="131" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="132" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="133" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="134" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="135" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="136" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="137" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="138" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="139" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="140" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="141" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="142" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="143" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="144" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="145" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="146" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="147" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="148" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="149" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="150" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="151" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="152" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="153" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="154" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="155" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="156" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="157" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="158" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="159" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="160" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="21" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="22" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="26" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="33" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="34" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="35" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="36" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="37" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="49" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="50" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="51" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="52" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="54" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="55" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="57" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="58" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="59" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="62" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="63" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="64" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="66" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="67" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="68" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="69" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="70" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="71" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="72" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="73" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="74" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="76" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="77" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="78" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="79" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="80" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="81" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="82" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="83" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="84" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="85" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="86" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="87" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="88" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="89" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="90" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="91" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="92" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="93" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="94" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="95" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="96" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="97" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="98" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="99" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="100" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="101" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="102" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="103" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="104" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="105" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="106" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="107" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="108" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="109" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="110" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="111" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="112" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="113" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="114" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="115" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="116" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="117" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="118" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="119" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="120" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="121" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="122" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="123" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="124" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="125" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="126" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="127" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="128" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="129" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="130" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="131" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="132" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="133" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="134" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="135" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="136" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="137" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="138" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="139" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="140" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="141" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="142" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="143" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="144" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="145" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="146" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="147" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="148" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="149" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="150" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="151" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="152" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="153" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="154" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="155" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="156" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="157" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="158" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="159" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="162" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="163" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="164" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="165" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="166" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="167" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="168" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="169" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="170" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="171" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="172" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="173" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="174" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="175" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="176" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="177" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="178" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="179" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="180" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="181" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="182" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="183" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="184" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="185" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="186" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="187" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="188" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="189" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="190" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="191" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="192" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="193" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="194" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="195" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="196" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="197" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="198" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="199" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="200" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="201" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="202" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="203" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="204" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="205" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="206" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="207" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="208" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="209" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="210" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="211" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="212" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="213" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="214" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="215" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="216" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="217" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="218" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="219" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="220" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="221" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="222" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="223" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="224" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="225" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="226" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="227" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="229" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="230" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="231" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="232" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="233" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="234" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="235" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="236" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="237" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="238" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="239" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="240" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="241" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="242" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="243" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="244" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="245" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="246" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="247" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="248" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="249" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="250" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="251" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="252" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="253" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="254" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="255" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="256" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="257" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="258" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="259" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="260" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="261" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="262" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="263" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="264" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="265" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="266" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="267" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="268" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="269" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="270" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="271" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="272" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="273" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="274" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="275" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="276" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="277" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="278" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="279" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="280" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="281" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="282" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="283" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="284" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="285" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="286" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="287" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="288" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="289" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="290" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="291" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="292" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="293" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="294" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="295" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="296" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="297" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="298" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="299" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="300" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="301" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="302" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="303" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="304" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="305" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="306" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="307" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="308" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="309" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="310" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="311" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="312" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="313" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="314" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="315" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="316" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="317" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="318" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="319" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="320" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="321" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="322" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="323" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="324" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="325" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="326" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="327" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="328" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="329" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="330" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="331" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="332" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="333" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="334" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="335" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="336" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="337" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="338" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="339" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="340" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="341" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="342" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="343" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="344" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="345" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="346" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="347" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="348" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="349" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="350" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="351" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="352" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="353" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="354" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="355" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="356" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="357" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="358" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="359" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="360" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="361" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="362" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="363" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="364" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="365" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="366" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="367" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="368" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="369" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="370" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="371" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="372" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="373" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="374" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="375" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="376" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="377" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="378" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="379" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="380" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="381" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="382" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="383" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="384" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="385" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="386" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="387" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="388" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="389" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="390" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="391" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="392" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="393" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="394" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="395" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="396" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="397" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="398" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="399" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="400" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="401" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="402" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="403" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="404" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="405" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="406" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="407" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="408" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="409" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="410" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="411" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="412" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="413" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="414" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="415" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="416" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="417" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="418" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="419" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="420" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="421" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="422" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="423" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="424" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="425" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="426" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="427" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="428" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="429" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="430" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="431" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="432" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="433" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="434" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="435" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="436" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="437" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="438" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="439" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="440" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="441" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="442" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="443" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="444" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="445" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="446" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="447" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="448" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="449" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="450" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="451" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="452" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="453" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="454" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="455" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="456" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="457" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="458" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="459" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="460" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="461" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="462" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="463" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="464" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="465" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="466" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="467" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="468" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="469" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="470" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="471" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="472" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="473" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="474" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="475" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="476" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="477" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="478" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="479" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="480" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="481" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="482" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="483" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="484" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="485" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="486" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="487" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="488" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="489" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="490" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="491" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="492" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="493" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="494" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="495" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="496" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="497" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="498" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="499" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="500" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="501" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="502" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="503" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="504" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="505" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="506" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="507" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="508" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="509" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="510" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="511" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="512" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="513" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="514" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="515" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="516" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="517" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="518" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="519" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="520" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="521" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="522" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="523" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="524" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="525" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="526" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="527" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="528" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="529" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="530" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="531" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="532" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="533" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="534" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="535" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="536" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="537" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="538" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="539" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="540" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="541" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="542" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="543" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="544" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="545" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="546" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="547" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="548" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="549" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="550" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="551" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="552" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="553" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="554" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="555" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="556" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="557" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="558" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="559" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="560" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="561" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="562" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="563" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="564" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="565" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="566" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="567" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="568" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="569" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="570" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="571" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="572" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="573" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="574" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="575" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="576" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="577" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="578" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="579" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="580" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="581" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="582" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="583" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="584" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="585" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="586" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="587" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="588" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="589" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="590" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="591" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="592" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="593" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="594" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="595" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="596" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="597" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="598" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="599" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="600" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="601" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="602" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="603" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="604" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="605" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="606" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="607" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="608" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="609" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="610" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="611" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="612" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="613" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="614" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="615" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="616" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="617" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="618" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="619" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="620" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="621" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="622" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="623" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="624" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="625" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="626" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="627" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="628" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="629" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="630" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="631" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="632" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="633" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="634" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="635" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="636" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="637" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="638" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="639" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="640" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="641" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="642" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="643" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="644" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="645" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="646" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="647" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="648" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="649" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="650" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="651" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="652" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="653" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="654" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="655" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="656" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="657" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="658" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="659" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="660" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="661" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="662" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="663" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="664" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="665" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="666" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="667" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="668" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="669" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="670" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="671" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="672" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="673" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="674" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="675" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="676" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="677" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="678" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="679" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="680" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="681" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="682" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="683" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="684" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="685" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="686" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="687" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="688" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="689" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="690" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="691" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="692" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="693" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="694" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="695" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="696" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="697" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="698" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="699" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="700" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="701" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="702" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="703" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="704" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="705" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="706" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="707" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="708" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="709" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="710" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="711" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="712" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="713" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="714" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="715" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="716" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="717" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="718" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="719" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="720" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="721" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="722" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="723" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="724" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="725" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="726" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="727" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="728" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="729" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="730" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="731" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="732" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="733" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="734" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="735" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="736" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="737" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="738" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="739" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="740" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="741" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="742" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="743" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="744" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="745" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="746" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="747" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="748" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="749" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="750" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="751" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="752" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="753" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="754" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="755" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="756" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="757" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="758" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="759" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="760" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="761" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="762" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="763" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="764" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="765" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="766" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="767" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="768" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="769" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="770" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="771" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="772" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="773" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="774" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="775" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="776" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="777" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="778" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="779" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="780" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="781" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="782" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="783" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="784" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="785" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="786" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="787" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="788" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="789" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="790" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="791" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="792" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="793" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="794" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="795" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="796" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="797" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="798" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="799" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="800" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="801" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="802" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="803" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="804" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="805" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="806" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="807" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="808" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="809" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="810" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="811" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="812" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="813" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="814" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="815" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="816" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="817" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="818" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="819" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="820" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="821" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="822" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="823" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="824" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="825" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="826" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="827" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="828" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="829" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="830" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="831" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="832" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="833" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="834" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="835" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="836" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="837" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="838" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="839" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="840" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="841" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="842" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="843" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="844" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="845" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="846" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="847" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="848" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="849" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="850" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="851" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="852" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="853" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="854" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="855" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="856" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="857" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="858" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="859" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="860" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="861" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="862" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="863" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="864" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="865" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="866" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="867" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="868" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="869" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="870" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="871" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="872" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="873" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="874" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="875" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="876" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="877" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="878" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="879" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="880" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="881" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="882" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="883" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="884" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="885" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="886" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="887" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="888" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="889" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="890" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="891" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="892" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="893" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="894" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="895" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="896" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="897" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="898" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="899" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="900" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="901" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="902" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="903" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="904" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="905" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="906" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="907" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="908" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="909" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="910" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="911" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="912" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="913" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="914" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="915" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="916" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="917" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="918" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="919" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="920" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="921" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="922" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="923" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="924" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="925" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="926" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="927" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="928" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="929" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="930" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="931" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="932" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="933" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="934" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="935" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="936" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="937" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="938" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="939" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="940" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="941" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="942" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="943" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="944" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="945" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="946" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="947" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="948" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="949" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="950" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="951" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="952" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="953" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="954" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="955" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="956" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="957" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="958" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="959" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="960" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="961" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="962" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="963" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="964" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="965" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="966" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="967" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="968" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="969" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="970" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="971" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="972" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="973" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="974" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="975" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="976" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="977" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="978" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="979" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="980" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="981" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="982" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="983" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="984" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="985" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="986" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="987" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="988" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="989" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="990" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="991" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="992" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="993" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="994" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="995" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="996" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="997" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="998" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="999" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1000" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -4357,13 +4367,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="C1" s="19" t="s">
         <v>49</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4371,10 +4381,10 @@
         <v>1001</v>
       </c>
       <c r="B2" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="20" t="s">
         <v>51</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4382,10 +4392,10 @@
         <v>1002</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4393,10 +4403,10 @@
         <v>1004</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4404,10 +4414,10 @@
         <v>1005</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4415,10 +4425,10 @@
         <v>1006</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4426,10 +4436,10 @@
         <v>1007</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4437,10 +4447,10 @@
         <v>1017</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4448,10 +4458,10 @@
         <v>1018</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4459,10 +4469,10 @@
         <v>2003</v>
       </c>
       <c r="B10" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="20" t="s">
         <v>60</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4470,10 +4480,10 @@
         <v>2005</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4481,10 +4491,10 @@
         <v>2008</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4492,10 +4502,10 @@
         <v>2009</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4503,10 +4513,10 @@
         <v>2011</v>
       </c>
       <c r="B14" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>65</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4514,10 +4524,10 @@
         <v>2014</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4525,10 +4535,10 @@
         <v>2016</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4536,10 +4546,10 @@
         <v>2018</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4547,10 +4557,10 @@
         <v>2022</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4558,10 +4568,10 @@
         <v>2025</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -4569,10 +4579,10 @@
         <v>2032</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4580,10 +4590,10 @@
         <v>2034</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4591,10 +4601,10 @@
         <v>2037</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4602,10 +4612,10 @@
         <v>4010</v>
       </c>
       <c r="B23" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="20" t="s">
         <v>75</v>
-      </c>
-      <c r="C23" s="20" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4613,10 +4623,10 @@
         <v>4017</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4624,10 +4634,10 @@
         <v>5006</v>
       </c>
       <c r="B25" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="20" t="s">
         <v>77</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4635,10 +4645,10 @@
         <v>5007</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4646,10 +4656,10 @@
         <v>5011</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
[feat/ASP-8019-report-parameters] Removed text wrapping for new cell
</commit_message>
<xml_diff>
--- a/api/templates/critical_errors_by_device/en.xlsx
+++ b/api/templates/critical_errors_by_device/en.xlsx
@@ -402,9 +402,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1" shrinkToFit="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -3229,7 +3227,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
-    <row r="5" ht="17" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" ht="17" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>

</xml_diff>